<commit_message>
Update race participant details in legal documents
</commit_message>
<xml_diff>
--- a/1_Kasim_2026_TT_Sampiyonasi_Hak_Kazananlar.xlsx
+++ b/1_Kasim_2026_TT_Sampiyonasi_Hak_Kazananlar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ktbf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51E822DB-2CFC-4DB2-A9D8-EDE64F9A3BFF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CAF83D1-EB58-48C5-966A-435D01461038}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4380" xr2:uid="{808AA03E-491F-4E19-9903-AA8B080AA830}"/>
   </bookViews>
@@ -1016,7 +1016,7 @@
         <v>24</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>12</v>
@@ -1025,7 +1025,7 @@
         <v>34</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
@@ -1033,16 +1033,16 @@
         <v>36</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -1050,7 +1050,7 @@
         <v>36</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>12</v>
@@ -1059,7 +1059,7 @@
         <v>9</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -1067,16 +1067,16 @@
         <v>36</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -1084,16 +1084,16 @@
         <v>36</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -1101,7 +1101,7 @@
         <v>36</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>12</v>
@@ -1110,7 +1110,7 @@
         <v>18</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -1118,16 +1118,16 @@
         <v>36</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>48</v>
+        <v>18</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
@@ -1135,16 +1135,16 @@
         <v>36</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
@@ -1152,7 +1152,7 @@
         <v>36</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>12</v>
@@ -1161,7 +1161,7 @@
         <v>51</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
@@ -1169,16 +1169,16 @@
         <v>36</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>